<commit_message>
Update F4 continuous maneuver outputs
</commit_message>
<xml_diff>
--- a/projects/F4/data/design_continuous_thrust_maneuver_strategy.xlsx
+++ b/projects/F4/data/design_continuous_thrust_maneuver_strategy.xlsx
@@ -152,34 +152,34 @@
         <v>0</v>
       </c>
       <c r="C2" s="2">
-        <v>1220.25517082</v>
+        <v>1214.07576963</v>
       </c>
       <c r="D2" s="2">
-        <v>1286.45770391</v>
+        <v>1282.04995367</v>
       </c>
       <c r="E2" s="2">
-        <v>3987.99652047</v>
+        <v>3967.60591505</v>
       </c>
       <c r="F2" s="2">
-        <v>4044.02039603</v>
+        <v>4022.65634789</v>
       </c>
       <c r="G2" s="2">
-        <v>7054.06898894</v>
+        <v>7010.49614755</v>
       </c>
       <c r="H2" s="2">
-        <v>7121.99562913</v>
+        <v>7084.06434862</v>
       </c>
       <c r="I2" s="2">
-        <v>9518.50043129</v>
+        <v>9525.38305607</v>
       </c>
       <c r="J2" s="2">
-        <v>9589.69379257</v>
+        <v>9590.2236564</v>
       </c>
       <c r="K2" s="2">
-        <v>10379.5235481</v>
+        <v>10379.1425282</v>
       </c>
       <c r="L2" s="2">
-        <v>10405.5954615</v>
+        <v>10404.8144827</v>
       </c>
     </row>
     <row r="3">
@@ -290,34 +290,34 @@
         <v>29478.137</v>
       </c>
       <c r="C5" s="2">
-        <v>29478.137</v>
+        <v>29371.3437044</v>
       </c>
       <c r="D5" s="2">
-        <v>31349.2007072</v>
+        <v>31241.1815907</v>
       </c>
       <c r="E5" s="2">
-        <v>31349.2007072</v>
+        <v>31241.1838887</v>
       </c>
       <c r="F5" s="2">
-        <v>33658.3972121</v>
+        <v>33512.8382243</v>
       </c>
       <c r="G5" s="2">
-        <v>33658.3972121</v>
+        <v>33512.8436363</v>
       </c>
       <c r="H5" s="2">
-        <v>38106.1296414</v>
+        <v>38548.6837017</v>
       </c>
       <c r="I5" s="2">
-        <v>38106.1296414</v>
+        <v>38548.6855854</v>
       </c>
       <c r="J5" s="2">
-        <v>47304.1761056</v>
+        <v>47196.1186129</v>
       </c>
       <c r="K5" s="2">
-        <v>47304.1761056</v>
+        <v>47196.7198857</v>
       </c>
       <c r="L5" s="2">
-        <v>42164.1999212</v>
+        <v>42164.1999818</v>
       </c>
     </row>
     <row r="6">
@@ -330,34 +330,34 @@
         <v>0.77684692</v>
       </c>
       <c r="C6" s="2">
-        <v>0.77684692</v>
+        <v>0.775921975106</v>
       </c>
       <c r="D6" s="2">
-        <v>0.67108772234</v>
+        <v>0.66995047829</v>
       </c>
       <c r="E6" s="2">
-        <v>0.67108772234</v>
+        <v>0.669950249593</v>
       </c>
       <c r="F6" s="2">
-        <v>0.556653039268</v>
+        <v>0.556957329964</v>
       </c>
       <c r="G6" s="2">
-        <v>0.556653039268</v>
+        <v>0.556957180195</v>
       </c>
       <c r="H6" s="2">
-        <v>0.375418285734</v>
+        <v>0.354157716447</v>
       </c>
       <c r="I6" s="2">
-        <v>0.375418285734</v>
+        <v>0.354157552399</v>
       </c>
       <c r="J6" s="2">
-        <v>0.10865797395</v>
+        <v>0.106617209294</v>
       </c>
       <c r="K6" s="2">
-        <v>0.10865797395</v>
+        <v>0.106676344957</v>
       </c>
       <c r="L6" s="2">
-        <v>0.000261954823015</v>
+        <v>0.000456170348255</v>
       </c>
     </row>
     <row r="7">
@@ -370,34 +370,34 @@
         <v>16.5</v>
       </c>
       <c r="C7" s="2">
-        <v>16.5</v>
+        <v>16.4986709821</v>
       </c>
       <c r="D7" s="2">
-        <v>12.9895109461</v>
+        <v>12.1957814767</v>
       </c>
       <c r="E7" s="2">
-        <v>12.9895109461</v>
+        <v>12.1958649194</v>
       </c>
       <c r="F7" s="2">
-        <v>10.2960066521</v>
+        <v>9.71745896517</v>
       </c>
       <c r="G7" s="2">
-        <v>10.2960066521</v>
+        <v>9.71752644059</v>
       </c>
       <c r="H7" s="2">
-        <v>7.40510985545</v>
+        <v>7.02289195997</v>
       </c>
       <c r="I7" s="2">
-        <v>7.40510985545</v>
+        <v>7.02293422062</v>
       </c>
       <c r="J7" s="2">
-        <v>6.00356177949</v>
+        <v>5.99941448567</v>
       </c>
       <c r="K7" s="2">
-        <v>6.00356177949</v>
+        <v>5.9994094242</v>
       </c>
       <c r="L7" s="2">
-        <v>6.00578523676</v>
+        <v>6.00193067629</v>
       </c>
     </row>
     <row r="8">
@@ -410,34 +410,34 @@
         <v>200</v>
       </c>
       <c r="C8" s="2">
-        <v>200.455057794</v>
+        <v>200.435319773</v>
       </c>
       <c r="D8" s="2">
-        <v>206.17207766</v>
+        <v>207.971441083</v>
       </c>
       <c r="E8" s="2">
-        <v>206.612489306</v>
+        <v>208.426092164</v>
       </c>
       <c r="F8" s="2">
-        <v>214.252923948</v>
+        <v>216.53977199</v>
       </c>
       <c r="G8" s="2">
-        <v>214.501642251</v>
+        <v>216.797387625</v>
       </c>
       <c r="H8" s="2">
-        <v>231.704490585</v>
+        <v>235.665788679</v>
       </c>
       <c r="I8" s="2">
-        <v>231.788914621</v>
+        <v>235.748085595</v>
       </c>
       <c r="J8" s="2">
-        <v>254.419732481</v>
+        <v>253.948400612</v>
       </c>
       <c r="K8" s="2">
-        <v>254.429669413</v>
+        <v>253.959040532</v>
       </c>
       <c r="L8" s="2">
-        <v>173.922720448</v>
+        <v>175.931423237</v>
       </c>
     </row>
     <row r="9">
@@ -450,34 +450,34 @@
         <v>8.53237</v>
       </c>
       <c r="C9" s="2">
-        <v>62.3907171836</v>
+        <v>63.9246175807</v>
       </c>
       <c r="D9" s="2">
-        <v>39.8229372108</v>
+        <v>39.0005992529</v>
       </c>
       <c r="E9" s="2">
-        <v>82.3600555718</v>
+        <v>85.5383357608</v>
       </c>
       <c r="F9" s="2">
-        <v>60.3899429051</v>
+        <v>63.3612285655</v>
       </c>
       <c r="G9" s="2">
-        <v>25.6900387869</v>
+        <v>34.224849418</v>
       </c>
       <c r="H9" s="2">
-        <v>350.895344856</v>
+        <v>356.312498094</v>
       </c>
       <c r="I9" s="2">
-        <v>110.08604353</v>
+        <v>104.270779373</v>
       </c>
       <c r="J9" s="2">
-        <v>67.2399854207</v>
+        <v>67.3153056945</v>
       </c>
       <c r="K9" s="2">
-        <v>229.236916257</v>
+        <v>229.540930727</v>
       </c>
       <c r="L9" s="2">
-        <v>222.769094702</v>
+        <v>223.182296756</v>
       </c>
     </row>
     <row r="10">
@@ -490,34 +490,34 @@
         <v>77.8161406659</v>
       </c>
       <c r="C10" s="2">
-        <v>77.5735175648</v>
+        <v>77.5583380045</v>
       </c>
       <c r="D10" s="2">
-        <v>71.601684997</v>
+        <v>69.6743924743</v>
       </c>
       <c r="E10" s="2">
-        <v>71.3726495961</v>
+        <v>69.4393215227</v>
       </c>
       <c r="F10" s="2">
-        <v>63.4468528912</v>
+        <v>61.0625033113</v>
       </c>
       <c r="G10" s="2">
-        <v>63.3194070476</v>
+        <v>60.931182709</v>
       </c>
       <c r="H10" s="2">
-        <v>45.5528674108</v>
+        <v>41.4612374173</v>
       </c>
       <c r="I10" s="2">
-        <v>45.5101198501</v>
+        <v>41.4202228899</v>
       </c>
       <c r="J10" s="2">
-        <v>20.5111323037</v>
+        <v>20.7192812153</v>
       </c>
       <c r="K10" s="2">
-        <v>20.5061225853</v>
+        <v>20.7146212909</v>
       </c>
       <c r="L10" s="2">
-        <v>20.5741250145</v>
+        <v>20.7915478086</v>
       </c>
     </row>
     <row r="11">
@@ -530,34 +530,34 @@
         <v>1.85437</v>
       </c>
       <c r="C11" s="2">
-        <v>165.285564853</v>
+        <v>165.357989945</v>
       </c>
       <c r="D11" s="2">
-        <v>192.615918598</v>
+        <v>193.603137297</v>
       </c>
       <c r="E11" s="2">
-        <v>169.142631551</v>
+        <v>169.184569361</v>
       </c>
       <c r="F11" s="2">
-        <v>190.171560507</v>
+        <v>189.958473423</v>
       </c>
       <c r="G11" s="2">
-        <v>168.250777822</v>
+        <v>166.993989366</v>
       </c>
       <c r="H11" s="2">
-        <v>190.659165964</v>
+        <v>191.210359525</v>
       </c>
       <c r="I11" s="2">
-        <v>169.942228744</v>
+        <v>171.310045027</v>
       </c>
       <c r="J11" s="2">
-        <v>190.33893459</v>
+        <v>190.081027023</v>
       </c>
       <c r="K11" s="2">
-        <v>356.963824397</v>
+        <v>357.083318165</v>
       </c>
       <c r="L11" s="2">
-        <v>83.3461737174</v>
+        <v>80.8951554821</v>
       </c>
     </row>
     <row r="12">
@@ -570,34 +570,34 @@
         <v>22.9025463458</v>
       </c>
       <c r="C12" s="2">
-        <v>177.05627882</v>
+        <v>177.062495201</v>
       </c>
       <c r="D12" s="2">
-        <v>183.357159079</v>
+        <v>183.631203309</v>
       </c>
       <c r="E12" s="2">
-        <v>177.112548496</v>
+        <v>177.115824747</v>
       </c>
       <c r="F12" s="2">
-        <v>183.492577779</v>
+        <v>183.417014494</v>
       </c>
       <c r="G12" s="2">
-        <v>175.963606318</v>
+        <v>175.532592063</v>
       </c>
       <c r="H12" s="2">
-        <v>185.231059339</v>
+        <v>185.727572117</v>
       </c>
       <c r="I12" s="2">
-        <v>175.064982688</v>
+        <v>175.56337805</v>
       </c>
       <c r="J12" s="2">
-        <v>188.369074729</v>
+        <v>188.191812309</v>
       </c>
       <c r="K12" s="2">
-        <v>356.201634491</v>
+        <v>356.366459516</v>
       </c>
       <c r="L12" s="2">
-        <v>83.3759904694</v>
+        <v>80.9467747834</v>
       </c>
     </row>
     <row r="13">
@@ -610,34 +610,34 @@
         <v>200.000064212</v>
       </c>
       <c r="C13" s="2">
-        <v>200.000064212</v>
+        <v>203.335685743</v>
       </c>
       <c r="D13" s="2">
-        <v>3933.00000741</v>
+        <v>3933.00004167</v>
       </c>
       <c r="E13" s="2">
-        <v>3933.00000741</v>
+        <v>3933.00794489</v>
       </c>
       <c r="F13" s="2">
-        <v>8544.21110711</v>
+        <v>8469.48032738</v>
       </c>
       <c r="G13" s="2">
-        <v>8544.21110711</v>
+        <v>8469.48774434</v>
       </c>
       <c r="H13" s="2">
-        <v>17422.2547755</v>
+        <v>18518.2329099</v>
       </c>
       <c r="I13" s="2">
-        <v>17422.2547755</v>
+        <v>18518.2404503</v>
       </c>
       <c r="J13" s="2">
-        <v>35786.0631706</v>
+        <v>35786.0631569</v>
       </c>
       <c r="K13" s="2">
-        <v>35786.0631706</v>
+        <v>35783.8093143</v>
       </c>
       <c r="L13" s="2">
-        <v>35775.0178057</v>
+        <v>35766.8289241</v>
       </c>
     </row>
     <row r="14">
@@ -650,34 +650,34 @@
         <v>45999.9999358</v>
       </c>
       <c r="C14" s="2">
-        <v>45999.9999358</v>
+        <v>45783.077723</v>
       </c>
       <c r="D14" s="2">
-        <v>46009.127407</v>
+        <v>45793.0891397</v>
       </c>
       <c r="E14" s="2">
-        <v>46009.127407</v>
+        <v>45793.0858325</v>
       </c>
       <c r="F14" s="2">
-        <v>46016.3093171</v>
+        <v>45799.9221212</v>
       </c>
       <c r="G14" s="2">
-        <v>46016.3093171</v>
+        <v>45799.9255283</v>
       </c>
       <c r="H14" s="2">
-        <v>46033.7305073</v>
+        <v>45822.8604935</v>
       </c>
       <c r="I14" s="2">
-        <v>46033.7305073</v>
+        <v>45822.8567206</v>
       </c>
       <c r="J14" s="2">
-        <v>46066.0150406</v>
+        <v>45849.900069</v>
       </c>
       <c r="K14" s="2">
-        <v>46066.0150406</v>
+        <v>45853.3564571</v>
       </c>
       <c r="L14" s="2">
-        <v>35797.1080367</v>
+        <v>35805.2970396</v>
       </c>
     </row>
     <row r="15">
@@ -693,31 +693,31 @@
         <v>6515</v>
       </c>
       <c r="D15" s="2">
-        <v>5909.34154485</v>
+        <v>5892.13926833</v>
       </c>
       <c r="E15" s="2">
-        <v>5909.34154485</v>
+        <v>5892.13926833</v>
       </c>
       <c r="F15" s="2">
-        <v>5402.51524476</v>
+        <v>5394.76484743</v>
       </c>
       <c r="G15" s="2">
-        <v>5402.51524476</v>
+        <v>5394.76484743</v>
       </c>
       <c r="H15" s="2">
-        <v>4780.11615163</v>
+        <v>4717.58764458</v>
       </c>
       <c r="I15" s="2">
-        <v>4780.11615163</v>
+        <v>4717.58764458</v>
       </c>
       <c r="J15" s="2">
-        <v>4125.99803422</v>
+        <v>4125.15320731</v>
       </c>
       <c r="K15" s="2">
-        <v>4125.99803422</v>
+        <v>4125.15320731</v>
       </c>
       <c r="L15" s="2">
-        <v>3909.99760767</v>
+        <v>3913.03627941</v>
       </c>
     </row>
     <row r="16">
@@ -730,34 +730,34 @@
         <v>-129.764366081</v>
       </c>
       <c r="C16" s="2">
-        <v>79.222505574</v>
+        <v>80.7434548773</v>
       </c>
       <c r="D16" s="2">
-        <v>68.7195232495</v>
+        <v>70.0225440835</v>
       </c>
       <c r="E16" s="2">
-        <v>105.542823266</v>
+        <v>110.575087537</v>
       </c>
       <c r="F16" s="2">
-        <v>97.686151689</v>
+        <v>102.910928031</v>
       </c>
       <c r="G16" s="2">
-        <v>55.7504253288</v>
+        <v>66.1818094185</v>
       </c>
       <c r="H16" s="2">
-        <v>47.6111143792</v>
+        <v>57.5241150293</v>
       </c>
       <c r="I16" s="2">
-        <v>156.700446239</v>
+        <v>155.371539164</v>
       </c>
       <c r="J16" s="2">
-        <v>149.989446042</v>
+        <v>149.412778603</v>
       </c>
       <c r="K16" s="2">
-        <v>119.769418373</v>
+        <v>119.766460801</v>
       </c>
       <c r="L16" s="2">
-        <v>119.999999909</v>
+        <v>119.990691906</v>
       </c>
     </row>
     <row r="17">
@@ -770,34 +770,34 @@
         <v>-11.148025327</v>
       </c>
       <c r="C17" s="2">
-        <v>4.90239979743</v>
+        <v>4.89833929662</v>
       </c>
       <c r="D17" s="2">
-        <v>6.36046399713</v>
+        <v>6.35577344324</v>
       </c>
       <c r="E17" s="2">
-        <v>5.18873681929</v>
+        <v>5.22613137452</v>
       </c>
       <c r="F17" s="2">
-        <v>6.28146302133</v>
+        <v>6.22299837908</v>
       </c>
       <c r="G17" s="2">
-        <v>5.19931974365</v>
+        <v>5.17905101712</v>
       </c>
       <c r="H17" s="2">
-        <v>6.20074140203</v>
+        <v>6.16203492599</v>
       </c>
       <c r="I17" s="2">
-        <v>5.39580215815</v>
+        <v>5.47640831121</v>
       </c>
       <c r="J17" s="2">
-        <v>5.95590231895</v>
+        <v>5.94285013048</v>
       </c>
       <c r="K17" s="2">
-        <v>-5.66263983975</v>
+        <v>-5.64799216439</v>
       </c>
       <c r="L17" s="2">
-        <v>-5.8583004356</v>
+        <v>-5.84466492961</v>
       </c>
     </row>
     <row r="18">
@@ -810,34 +810,34 @@
         <v>839.478889761</v>
       </c>
       <c r="C18" s="2">
-        <v>839.478889761</v>
+        <v>834.921132011</v>
       </c>
       <c r="D18" s="2">
-        <v>920.660347458</v>
+        <v>915.906006102</v>
       </c>
       <c r="E18" s="2">
-        <v>920.660347458</v>
+        <v>915.906107159</v>
       </c>
       <c r="F18" s="2">
-        <v>1024.23562436</v>
+        <v>1017.59870408</v>
       </c>
       <c r="G18" s="2">
-        <v>1024.23562436</v>
+        <v>1017.59895058</v>
       </c>
       <c r="H18" s="2">
-        <v>1233.82052637</v>
+        <v>1255.37668808</v>
       </c>
       <c r="I18" s="2">
-        <v>1233.82052637</v>
+        <v>1255.3767801</v>
       </c>
       <c r="J18" s="2">
-        <v>1706.5104588</v>
+        <v>1700.6664961</v>
       </c>
       <c r="K18" s="2">
-        <v>1706.5104588</v>
+        <v>1700.69899563</v>
       </c>
       <c r="L18" s="2">
-        <v>1436.06972283</v>
+        <v>1436.06972593</v>
       </c>
     </row>
     <row r="19">
@@ -850,34 +850,34 @@
         <v>149.555673284</v>
       </c>
       <c r="C19" s="2">
-        <v>149.555673284</v>
+        <v>150.698232404</v>
       </c>
       <c r="D19" s="2">
-        <v>129.204741992</v>
+        <v>130.39658157</v>
       </c>
       <c r="E19" s="2">
-        <v>129.204741992</v>
+        <v>130.396556237</v>
       </c>
       <c r="F19" s="2">
-        <v>103.240027836</v>
+        <v>104.903800728</v>
       </c>
       <c r="G19" s="2">
-        <v>103.240027836</v>
+        <v>104.903738934</v>
       </c>
       <c r="H19" s="2">
-        <v>50.7003462192</v>
+        <v>45.296551086</v>
       </c>
       <c r="I19" s="2">
-        <v>50.7003462192</v>
+        <v>45.2965280186</v>
       </c>
       <c r="J19" s="2">
-        <v>-67.7956824351</v>
+        <v>-66.3306917007</v>
       </c>
       <c r="K19" s="2">
-        <v>-67.7956824351</v>
+        <v>-66.3388388274</v>
       </c>
       <c r="L19" s="2">
-        <v>-0.000387888785212</v>
+        <v>-0.000388665300534</v>
       </c>
     </row>
     <row r="20">
@@ -892,23 +892,23 @@
         </is>
       </c>
       <c r="C20" s="2">
-        <v>5.46975159268</v>
+        <v>10</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2">
-        <v>10.0742422839</v>
+        <v>10</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2">
-        <v>15.4800186428</v>
+        <v>14</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2">
-        <v>14.5905383569</v>
+        <v>12.7326328892</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2">
-        <v>-178.537753748</v>
+        <v>-178.523769161</v>
       </c>
       <c r="L20" s="2"/>
     </row>
@@ -924,23 +924,23 @@
         </is>
       </c>
       <c r="C21" s="2">
-        <v>605.658455152</v>
+        <v>622.860731668</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2">
-        <v>506.826300086</v>
+        <v>497.374420906</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2">
-        <v>622.399093136</v>
+        <v>677.177202844</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2">
-        <v>654.118117406</v>
+        <v>592.434437273</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2">
-        <v>216.000426555</v>
+        <v>212.1169279</v>
       </c>
       <c r="L21" s="2"/>
     </row>
@@ -956,23 +956,23 @@
         </is>
       </c>
       <c r="C22" s="2">
-        <v>295.353255012</v>
+        <v>304.179165745</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2">
-        <v>271.418592475</v>
+        <v>266.938781249</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2">
-        <v>370.496295541</v>
+        <v>406.012170488</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2">
-        <v>445.428382819</v>
+        <v>406.185226113</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2">
-        <v>162.705240645</v>
+        <v>159.733512236</v>
       </c>
       <c r="L22" s="2"/>
     </row>
@@ -988,23 +988,23 @@
         </is>
       </c>
       <c r="C23" s="2">
-        <v>66.2025330861</v>
+        <v>67.9741840363</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2">
-        <v>56.0238755544</v>
+        <v>55.050432841</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2">
-        <v>67.9266401927</v>
+        <v>73.5682010651</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2">
-        <v>71.1933612823</v>
+        <v>64.8406003316</v>
       </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2">
-        <v>26.0719134013</v>
+        <v>25.6719544729</v>
       </c>
       <c r="L23" s="2"/>
     </row>
@@ -1052,23 +1052,23 @@
         </is>
       </c>
       <c r="C25" s="2">
-        <v>62.2025330861</v>
+        <v>63.9741840363</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2">
-        <v>52.0238755544</v>
+        <v>51.050432841</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2">
-        <v>63.9266401927</v>
+        <v>69.5682010651</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2">
-        <v>67.1933612823</v>
+        <v>60.8406003316</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2">
-        <v>22.0719134013</v>
+        <v>21.6719544729</v>
       </c>
       <c r="L25" s="2"/>
     </row>

</xml_diff>